<commit_message>
Fix RF training bug, Update forecast plot, add project pdf
</commit_message>
<xml_diff>
--- a/Inflation rates from bsp.xlsx
+++ b/Inflation rates from bsp.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marry Bless Magat\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marry Bless Magat\Documents\lenon files\Projects\ARIMA_RF Model Python Version\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA83F856-A879-4FF1-BD1D-1D8A52E657B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68EA598C-4700-4CF5-ABE2-62F5227C21C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{E0724E5E-9433-4F78-8797-5AA96C5BE9E8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E0724E5E-9433-4F78-8797-5AA96C5BE9E8}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>